<commit_message>
Build cross-platform pipeline and content intake workflow
</commit_message>
<xml_diff>
--- a/CNPA URLS and opinion feeds.xlsx
+++ b/CNPA URLS and opinion feeds.xlsx
@@ -1,13 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="CNPA URLS and opinion feeds" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Codex</Application>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Codex</dc:creator>
+  <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-04-14T23:19:52Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-04-14T23:19:52Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="2">
     <font>
@@ -47,7 +54,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="CNPA URLS and opinion feeds" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L336"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -245,7 +260,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -304,7 +319,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -533,7 +548,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gold Mountian Media</t>
+          <t>Gold Mountain California News Media Inc. (GMCNMI)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -565,7 +580,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -597,7 +612,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Alden Global Capital</t>
+          <t>MediaNews Group</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -922,7 +937,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1782,7 +1797,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Appeal-Democrat (A-D)</t>
+          <t>Glen County Transcript</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1986,7 +2001,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Los Angeles Times Communications LLC (LATCLLC)</t>
+          <t>Times Community News</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2114,7 +2129,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Sound California News Media Inc. (SCNMI)</t>
+          <t>Tehachapi News</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2889,7 +2904,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Big Bear Grizzly</t>
+          <t>Gold Mountain California News Media Inc. (GMCNMI)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3423,7 +3438,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Latino Media Collaborative</t>
+          <t>Impremedia</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3819,7 +3834,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Metropolitan News-Enterprise</t>
+          <t>Metropolitan News Company</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4316,7 +4331,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>McClatchy Papers</t>
+          <t>Chatham Asset Management (CAM)</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4385,7 +4400,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>The Sun-Gazette</t>
+          <t>Mineral King Publishing, Inc. (MKPI)</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -4498,7 +4513,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -4648,7 +4663,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Embarcadero Media Foundation (EMF)</t>
+          <t>Palo Alto Weekly</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -4931,7 +4946,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>The Sonoma Index-Tribune</t>
+          <t>MediaNews Group</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -5054,7 +5069,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Manteca/Ripon Bulletin</t>
+          <t>209 Multimedia</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -5123,7 +5138,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -5268,7 +5283,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Half Moon Bay Review</t>
+          <t>Coastside News Group, Inc. (CNGI)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -5465,7 +5480,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -5795,7 +5810,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>MediaNews Group</t>
+          <t>The San Diego Union-Tribune</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -5977,7 +5992,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Manteca/Ripon Bulletin</t>
+          <t>209 Multimedia</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -6036,7 +6051,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -6255,7 +6270,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -7861,7 +7876,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Embarcadero Media Foundation (EMF)</t>
+          <t>Palo Alto Weekly</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -8043,7 +8058,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>MediaNews Group</t>
+          <t>TIMES MEDIA GROUP (TMG)</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -8252,7 +8267,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Big Bear Grizzly</t>
+          <t>Gold Mountain California News Media Inc. (GMCNMI)</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -8311,7 +8326,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Manteca/Ripon Bulletin</t>
+          <t>209 Multimedia</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -9473,7 +9488,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>McClatchy Papers</t>
+          <t>Chatham Asset Management (CAM)</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -9645,7 +9660,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Hoffmann Media Group</t>
+          <t>Napa Valley Register</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -9677,7 +9692,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Turlock Journal</t>
+          <t>209 Multimedia</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -9970,7 +9985,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Visalia Times-Delta</t>
+          <t>Gannett Company Inc. (GCI)</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -10157,7 +10172,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>McClatchy Papers</t>
+          <t>Chatham Asset Management (CAM)</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -10344,7 +10359,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>HLR Media, LLC (HLRM-VR)</t>
+          <t>Beacon Media, Inc. (BMI-VR)</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">

</xml_diff>